<commit_message>
Mover plantilla de horas extras a public
</commit_message>
<xml_diff>
--- a/public/plantilla-horas-extra.xlsx
+++ b/public/plantilla-horas-extra.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Gerencia A&amp;D\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\proyecto\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{0E1E18B2-795A-4793-AF3E-A7833027A721}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1187BD18-1D69-48E8-B675-540339B74926}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{44F16EB2-3180-4466-BB78-D60D707A8425}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="49">
   <si>
     <t>FORMULARIO DE SOLICITUD DE HORAS EXTRAS</t>
   </si>
@@ -93,40 +93,94 @@
     <t xml:space="preserve">TOTAL DE PERSONAS: </t>
   </si>
   <si>
+    <t xml:space="preserve">Una vez finalizados los trabajos y cuando regresa el personal a la oficina, el responsible de realizar el o los trabajos deberá anotar la información indicada en el cuadro "Reporte de horas extras" con el fin de dar FE de las horas reales utilizadas que se requirieron para realizar los trabajos. </t>
+  </si>
+  <si>
+    <t>REPORTE DE HORAS EXTRAS</t>
+  </si>
+  <si>
+    <t>PROYECTO:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CLIENTE: </t>
+  </si>
+  <si>
+    <t xml:space="preserve">FECHA DE INICIO: </t>
+  </si>
+  <si>
+    <t xml:space="preserve">FECHA FINALIZACION: </t>
+  </si>
+  <si>
+    <t xml:space="preserve">SE CONFIRMA QUE LAS HORAS SOLICITADAS SON CORRECTAS: </t>
+  </si>
+  <si>
+    <t xml:space="preserve">SE CONFIRMA CANTIDAD DE PERSONAS: </t>
+  </si>
+  <si>
+    <t xml:space="preserve">MEDIO DE TRANSPORTE: </t>
+  </si>
+  <si>
+    <t>UBER</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VEHICULO DE SALVAVIDAS </t>
+  </si>
+  <si>
+    <t>KM</t>
+  </si>
+  <si>
+    <t>SI</t>
+  </si>
+  <si>
+    <t>(Marque la casilla correspondiente)</t>
+  </si>
+  <si>
+    <t>N/A</t>
+  </si>
+  <si>
+    <t>VEHICULO PERSONAL</t>
+  </si>
+  <si>
+    <t>NO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">COMENTARIOS ADICIONALES: </t>
+  </si>
+  <si>
+    <t xml:space="preserve">NOMBRE RESPONSABLE: </t>
+  </si>
+  <si>
+    <t xml:space="preserve">DEPARTAMENTO: </t>
+  </si>
+  <si>
+    <t>FINANZAS &amp; CONTABILIDAD</t>
+  </si>
+  <si>
+    <t>FIRMA:</t>
+  </si>
+  <si>
+    <t>ALARMA &amp; DETECCION</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Una vez finalizados los trabajos y cuando el personal regresa a la oficina (si aplica), el responsible de el o los trabajos deberá llenar esta información con el fin de dar FE de las horas reales utilizadas que se requirieron para realizar los trabajos en horario extra y bajo el entendido que Salvavidas tiene derecho a verificar por medio del tipo de transporte asignado que la información y horarios indicados son correctos. </t>
+  </si>
+  <si>
+    <t>INGENIERIA</t>
+  </si>
+  <si>
+    <t>LOGISTICA</t>
+  </si>
+  <si>
+    <t>MANTENIMIENTO</t>
+  </si>
+  <si>
+    <t>PROYECTOS</t>
+  </si>
+  <si>
     <t>RECURSOS HUMANOS</t>
   </si>
   <si>
     <t>VENTAS</t>
-  </si>
-  <si>
-    <t>Cristhian Espinoza</t>
-  </si>
-  <si>
-    <t>Instalacion</t>
-  </si>
-  <si>
-    <t>Supervisor</t>
-  </si>
-  <si>
-    <t>Zollner</t>
-  </si>
-  <si>
-    <t>A26A004</t>
-  </si>
-  <si>
-    <t>Jose Andres Melendez</t>
-  </si>
-  <si>
-    <t>Jeffry Marin</t>
-  </si>
-  <si>
-    <t>Operario</t>
-  </si>
-  <si>
-    <t>Angel Jiron</t>
-  </si>
-  <si>
-    <t>ayudante</t>
   </si>
 </sst>
 </file>
@@ -138,7 +192,7 @@
     <numFmt numFmtId="165" formatCode="[$-409]d\-mmm;@"/>
     <numFmt numFmtId="166" formatCode="#,##0.00\ &quot;hrs&quot;"/>
   </numFmts>
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -198,8 +252,15 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="18"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -218,8 +279,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.14999847407452621"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="22">
+  <borders count="41">
     <border>
       <left/>
       <right/>
@@ -510,11 +577,208 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="dashDot">
+        <color auto="1"/>
+      </top>
+      <bottom style="dashDot">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="hair">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="hair">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="hair">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="hair">
+        <color indexed="64"/>
+      </top>
+      <bottom style="hair">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="hair">
+        <color indexed="64"/>
+      </top>
+      <bottom style="hair">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="hair">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="dashDot">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="dashDot">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="dashDot">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="43">
+  <cellXfs count="87">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -563,23 +827,99 @@
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="34" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="35" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="35" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="36" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="37" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="37" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="38" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyProtection="1">
       <protection locked="0"/>
@@ -597,8 +937,43 @@
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="3" borderId="15" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
     </xf>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
@@ -628,6 +1003,15 @@
       <alignment horizontal="left"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
       <protection locked="0"/>
@@ -658,6 +1042,16 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="4" borderId="15" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="4" borderId="20" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="4" borderId="19" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
   </cellXfs>
@@ -695,20 +1089,80 @@
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>371474</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>87187</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>95465</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>10987</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print">
+          <a:clrChange>
+            <a:clrFrom>
+              <a:srgbClr val="FEFEFE"/>
+            </a:clrFrom>
+            <a:clrTo>
+              <a:srgbClr val="FEFEFE">
+                <a:alpha val="0"/>
+              </a:srgbClr>
+            </a:clrTo>
+          </a:clrChange>
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4038599" y="277687"/>
+          <a:ext cx="2067141" cy="1066800"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
       <xdr:twoCellAnchor editAs="oneCell">
         <xdr:from>
           <xdr:col>6</xdr:col>
           <xdr:colOff>289560</xdr:colOff>
-          <xdr:row>35</xdr:row>
-          <xdr:rowOff>0</xdr:rowOff>
+          <xdr:row>49</xdr:row>
+          <xdr:rowOff>182880</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>6</xdr:col>
           <xdr:colOff>533400</xdr:colOff>
-          <xdr:row>36</xdr:row>
-          <xdr:rowOff>53340</xdr:rowOff>
+          <xdr:row>51</xdr:row>
+          <xdr:rowOff>38100</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -768,14 +1222,14 @@
         <xdr:from>
           <xdr:col>6</xdr:col>
           <xdr:colOff>289560</xdr:colOff>
-          <xdr:row>35</xdr:row>
-          <xdr:rowOff>0</xdr:rowOff>
+          <xdr:row>50</xdr:row>
+          <xdr:rowOff>190500</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>6</xdr:col>
           <xdr:colOff>533400</xdr:colOff>
-          <xdr:row>36</xdr:row>
-          <xdr:rowOff>53340</xdr:rowOff>
+          <xdr:row>52</xdr:row>
+          <xdr:rowOff>45720</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -835,14 +1289,14 @@
         <xdr:from>
           <xdr:col>10</xdr:col>
           <xdr:colOff>251460</xdr:colOff>
-          <xdr:row>35</xdr:row>
-          <xdr:rowOff>0</xdr:rowOff>
+          <xdr:row>49</xdr:row>
+          <xdr:rowOff>190500</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>10</xdr:col>
           <xdr:colOff>495300</xdr:colOff>
-          <xdr:row>36</xdr:row>
-          <xdr:rowOff>45720</xdr:rowOff>
+          <xdr:row>51</xdr:row>
+          <xdr:rowOff>38100</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -902,14 +1356,14 @@
         <xdr:from>
           <xdr:col>10</xdr:col>
           <xdr:colOff>251460</xdr:colOff>
-          <xdr:row>35</xdr:row>
+          <xdr:row>51</xdr:row>
           <xdr:rowOff>0</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>10</xdr:col>
           <xdr:colOff>495300</xdr:colOff>
-          <xdr:row>36</xdr:row>
-          <xdr:rowOff>45720</xdr:rowOff>
+          <xdr:row>52</xdr:row>
+          <xdr:rowOff>38100</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -1263,7 +1717,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8540595A-1587-42A1-8DD0-E196AD6407A5}">
-  <dimension ref="B2:R37"/>
+  <dimension ref="B2:R68"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9.109375" style="4"/>
@@ -1377,21 +1831,21 @@
       <c r="O10" s="1"/>
     </row>
     <row r="11" spans="3:16" customFormat="1" ht="29.4" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="C11" s="39" t="s">
+      <c r="C11" s="80" t="s">
         <v>0</v>
       </c>
-      <c r="D11" s="40"/>
-      <c r="E11" s="40"/>
-      <c r="F11" s="40"/>
-      <c r="G11" s="40"/>
-      <c r="H11" s="40"/>
-      <c r="I11" s="40"/>
-      <c r="J11" s="40"/>
-      <c r="K11" s="40"/>
-      <c r="L11" s="40"/>
-      <c r="M11" s="40"/>
-      <c r="N11" s="40"/>
-      <c r="O11" s="41"/>
+      <c r="D11" s="81"/>
+      <c r="E11" s="81"/>
+      <c r="F11" s="81"/>
+      <c r="G11" s="81"/>
+      <c r="H11" s="81"/>
+      <c r="I11" s="81"/>
+      <c r="J11" s="81"/>
+      <c r="K11" s="81"/>
+      <c r="L11" s="81"/>
+      <c r="M11" s="81"/>
+      <c r="N11" s="81"/>
+      <c r="O11" s="82"/>
     </row>
     <row r="12" spans="3:16" customFormat="1" ht="15.9" customHeight="1" x14ac:dyDescent="0.4">
       <c r="C12" s="3"/>
@@ -1424,118 +1878,108 @@
       <c r="O13" s="3"/>
     </row>
     <row r="14" spans="3:16" ht="15.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C14" s="34" t="s">
+      <c r="C14" s="75" t="s">
         <v>1</v>
       </c>
-      <c r="D14" s="34"/>
-      <c r="E14" s="42" t="s">
-        <v>21</v>
-      </c>
-      <c r="F14" s="42"/>
-      <c r="G14" s="42"/>
-      <c r="H14" s="42"/>
-      <c r="I14" s="42"/>
-      <c r="J14" s="42"/>
-      <c r="K14" s="42"/>
-      <c r="L14" s="42"/>
-      <c r="M14" s="42"/>
-      <c r="N14" s="42"/>
-      <c r="O14" s="42"/>
+      <c r="D14" s="75"/>
+      <c r="E14" s="83"/>
+      <c r="F14" s="83"/>
+      <c r="G14" s="83"/>
+      <c r="H14" s="83"/>
+      <c r="I14" s="83"/>
+      <c r="J14" s="83"/>
+      <c r="K14" s="83"/>
+      <c r="L14" s="83"/>
+      <c r="M14" s="83"/>
+      <c r="N14" s="83"/>
+      <c r="O14" s="83"/>
     </row>
     <row r="15" spans="3:16" ht="15.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C15" s="34" t="s">
+      <c r="C15" s="75" t="s">
         <v>2</v>
       </c>
-      <c r="D15" s="34"/>
-      <c r="E15" s="26">
-        <v>46196</v>
-      </c>
-      <c r="F15" s="26"/>
-      <c r="G15" s="26"/>
-      <c r="H15" s="26"/>
-      <c r="I15" s="26"/>
-      <c r="J15" s="26"/>
-      <c r="K15" s="26"/>
-      <c r="L15" s="26"/>
-      <c r="M15" s="26"/>
-      <c r="N15" s="26"/>
-      <c r="O15" s="26"/>
+      <c r="D15" s="75"/>
+      <c r="E15" s="64"/>
+      <c r="F15" s="64"/>
+      <c r="G15" s="64"/>
+      <c r="H15" s="64"/>
+      <c r="I15" s="64"/>
+      <c r="J15" s="64"/>
+      <c r="K15" s="64"/>
+      <c r="L15" s="64"/>
+      <c r="M15" s="64"/>
+      <c r="N15" s="64"/>
+      <c r="O15" s="64"/>
     </row>
     <row r="16" spans="3:16" ht="15.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C16" s="34" t="s">
+      <c r="C16" s="75" t="s">
         <v>3</v>
       </c>
-      <c r="D16" s="34"/>
-      <c r="E16" s="33" t="s">
-        <v>24</v>
-      </c>
-      <c r="F16" s="33"/>
-      <c r="G16" s="33"/>
-      <c r="H16" s="33"/>
-      <c r="I16" s="33"/>
-      <c r="J16" s="33"/>
-      <c r="K16" s="33"/>
-      <c r="L16" s="33"/>
-      <c r="M16" s="33"/>
-      <c r="N16" s="33"/>
-      <c r="O16" s="33"/>
+      <c r="D16" s="75"/>
+      <c r="E16" s="74"/>
+      <c r="F16" s="74"/>
+      <c r="G16" s="74"/>
+      <c r="H16" s="74"/>
+      <c r="I16" s="74"/>
+      <c r="J16" s="74"/>
+      <c r="K16" s="74"/>
+      <c r="L16" s="74"/>
+      <c r="M16" s="74"/>
+      <c r="N16" s="74"/>
+      <c r="O16" s="74"/>
     </row>
     <row r="17" spans="2:16" ht="15.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C17" s="34" t="s">
+      <c r="C17" s="75" t="s">
         <v>4</v>
       </c>
-      <c r="D17" s="34"/>
-      <c r="E17" s="33" t="s">
-        <v>25</v>
-      </c>
-      <c r="F17" s="33"/>
-      <c r="G17" s="33"/>
-      <c r="H17" s="33"/>
-      <c r="I17" s="33"/>
-      <c r="J17" s="33"/>
-      <c r="K17" s="33"/>
-      <c r="L17" s="33"/>
-      <c r="M17" s="33"/>
-      <c r="N17" s="33"/>
-      <c r="O17" s="33"/>
+      <c r="D17" s="75"/>
+      <c r="E17" s="74"/>
+      <c r="F17" s="74"/>
+      <c r="G17" s="74"/>
+      <c r="H17" s="74"/>
+      <c r="I17" s="74"/>
+      <c r="J17" s="74"/>
+      <c r="K17" s="74"/>
+      <c r="L17" s="74"/>
+      <c r="M17" s="74"/>
+      <c r="N17" s="74"/>
+      <c r="O17" s="74"/>
     </row>
     <row r="18" spans="2:16" ht="15.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C18" s="35" t="s">
+      <c r="C18" s="76" t="s">
         <v>5</v>
       </c>
-      <c r="D18" s="35"/>
+      <c r="D18" s="76"/>
     </row>
     <row r="19" spans="2:16" ht="15.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C19" s="35"/>
-      <c r="D19" s="35"/>
-      <c r="E19" s="33" t="s">
-        <v>22</v>
-      </c>
-      <c r="F19" s="33"/>
-      <c r="G19" s="33"/>
-      <c r="H19" s="33"/>
-      <c r="I19" s="33"/>
-      <c r="J19" s="33"/>
-      <c r="K19" s="33"/>
-      <c r="L19" s="33"/>
-      <c r="M19" s="33"/>
-      <c r="N19" s="33"/>
-      <c r="O19" s="33"/>
+      <c r="C19" s="76"/>
+      <c r="D19" s="76"/>
+      <c r="E19" s="74"/>
+      <c r="F19" s="74"/>
+      <c r="G19" s="74"/>
+      <c r="H19" s="74"/>
+      <c r="I19" s="74"/>
+      <c r="J19" s="74"/>
+      <c r="K19" s="74"/>
+      <c r="L19" s="74"/>
+      <c r="M19" s="74"/>
+      <c r="N19" s="74"/>
+      <c r="O19" s="74"/>
     </row>
     <row r="20" spans="2:16" ht="15.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C20"/>
       <c r="D20"/>
-      <c r="E20" s="33"/>
-      <c r="F20" s="33"/>
-      <c r="G20" s="33"/>
-      <c r="H20" s="33"/>
-      <c r="I20" s="33"/>
-      <c r="J20" s="33"/>
-      <c r="K20" s="33"/>
-      <c r="L20" s="33"/>
-      <c r="M20" s="33"/>
-      <c r="N20" s="33"/>
-      <c r="O20" s="33"/>
+      <c r="E20" s="74"/>
+      <c r="F20" s="74"/>
+      <c r="G20" s="74"/>
+      <c r="H20" s="74"/>
+      <c r="I20" s="74"/>
+      <c r="J20" s="74"/>
+      <c r="K20" s="74"/>
+      <c r="L20" s="74"/>
+      <c r="M20" s="74"/>
+      <c r="N20" s="74"/>
+      <c r="O20" s="74"/>
     </row>
     <row r="21" spans="2:16" customFormat="1" ht="15.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="G21" s="1"/>
@@ -1549,36 +1993,36 @@
       <c r="O21" s="1"/>
     </row>
     <row r="22" spans="2:16" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="C22" s="36" t="s">
+      <c r="C22" s="77" t="s">
         <v>6</v>
       </c>
-      <c r="D22" s="36"/>
-      <c r="E22" s="36"/>
-      <c r="F22" s="36"/>
-      <c r="G22" s="36"/>
-      <c r="H22" s="36"/>
-      <c r="I22" s="36"/>
-      <c r="J22" s="36"/>
-      <c r="K22" s="36"/>
-      <c r="L22" s="36"/>
-      <c r="M22" s="36"/>
-      <c r="N22" s="36"/>
-      <c r="O22" s="36"/>
+      <c r="D22" s="77"/>
+      <c r="E22" s="77"/>
+      <c r="F22" s="77"/>
+      <c r="G22" s="77"/>
+      <c r="H22" s="77"/>
+      <c r="I22" s="77"/>
+      <c r="J22" s="77"/>
+      <c r="K22" s="77"/>
+      <c r="L22" s="77"/>
+      <c r="M22" s="77"/>
+      <c r="N22" s="77"/>
+      <c r="O22" s="77"/>
     </row>
     <row r="23" spans="2:16" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="C23" s="36"/>
-      <c r="D23" s="36"/>
-      <c r="E23" s="36"/>
-      <c r="F23" s="36"/>
-      <c r="G23" s="36"/>
-      <c r="H23" s="36"/>
-      <c r="I23" s="36"/>
-      <c r="J23" s="36"/>
-      <c r="K23" s="36"/>
-      <c r="L23" s="36"/>
-      <c r="M23" s="36"/>
-      <c r="N23" s="36"/>
-      <c r="O23" s="36"/>
+      <c r="C23" s="77"/>
+      <c r="D23" s="77"/>
+      <c r="E23" s="77"/>
+      <c r="F23" s="77"/>
+      <c r="G23" s="77"/>
+      <c r="H23" s="77"/>
+      <c r="I23" s="77"/>
+      <c r="J23" s="77"/>
+      <c r="K23" s="77"/>
+      <c r="L23" s="77"/>
+      <c r="M23" s="77"/>
+      <c r="N23" s="77"/>
+      <c r="O23" s="77"/>
     </row>
     <row r="24" spans="2:16" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="G24" s="1"/>
@@ -1606,10 +2050,10 @@
       <c r="O24" s="1"/>
     </row>
     <row r="25" spans="2:16" s="11" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="C25" s="37" t="s">
+      <c r="C25" s="78" t="s">
         <v>13</v>
       </c>
-      <c r="D25" s="38"/>
+      <c r="D25" s="79"/>
       <c r="E25" s="7" t="s">
         <v>14</v>
       </c>
@@ -1644,180 +2088,120 @@
         <v>17</v>
       </c>
     </row>
-    <row r="26" spans="2:16" s="20" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="B26" s="21"/>
-      <c r="C26" s="29" t="s">
-        <v>26</v>
-      </c>
-      <c r="D26" s="30"/>
-      <c r="E26" s="22" t="s">
-        <v>23</v>
-      </c>
-      <c r="F26" s="23">
-        <v>0.27083333333333331</v>
-      </c>
-      <c r="G26" s="23">
-        <v>0.29166666666666669</v>
-      </c>
-      <c r="H26" s="24"/>
-      <c r="I26" s="24"/>
-      <c r="J26" s="24"/>
-      <c r="K26" s="24">
-        <v>0.5</v>
-      </c>
-      <c r="L26" s="24"/>
-      <c r="M26" s="24"/>
-      <c r="N26" s="24"/>
-      <c r="O26" s="25">
+    <row r="26" spans="2:16" s="47" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="B26" s="48"/>
+      <c r="C26" s="67"/>
+      <c r="D26" s="68"/>
+      <c r="E26" s="49"/>
+      <c r="F26" s="50"/>
+      <c r="G26" s="50"/>
+      <c r="H26" s="51"/>
+      <c r="I26" s="51"/>
+      <c r="J26" s="51"/>
+      <c r="K26" s="51"/>
+      <c r="L26" s="51"/>
+      <c r="M26" s="51"/>
+      <c r="N26" s="51"/>
+      <c r="O26" s="84">
         <f>+SUM(H26:N26)</f>
-        <v>0.5</v>
-      </c>
-      <c r="P26" s="21"/>
+        <v>0</v>
+      </c>
+      <c r="P26" s="48"/>
     </row>
     <row r="27" spans="2:16" x14ac:dyDescent="0.3">
-      <c r="C27" s="27" t="s">
-        <v>26</v>
-      </c>
-      <c r="D27" s="28"/>
-      <c r="E27" s="12" t="s">
-        <v>23</v>
-      </c>
-      <c r="F27" s="13">
-        <v>0.6875</v>
-      </c>
-      <c r="G27" s="13">
-        <v>0.75</v>
-      </c>
+      <c r="C27" s="65"/>
+      <c r="D27" s="66"/>
+      <c r="E27" s="12"/>
+      <c r="F27" s="13"/>
+      <c r="G27" s="13"/>
       <c r="H27" s="14"/>
       <c r="I27" s="14"/>
       <c r="J27" s="14"/>
-      <c r="K27" s="14">
-        <v>1.5</v>
-      </c>
+      <c r="K27" s="14"/>
       <c r="L27" s="14"/>
       <c r="M27" s="14"/>
       <c r="N27" s="14"/>
-      <c r="O27" s="15">
+      <c r="O27" s="84">
         <f t="shared" ref="O27:O33" si="0">+SUM(H27:N27)</f>
-        <v>1.5</v>
-      </c>
-    </row>
-    <row r="28" spans="2:16" s="20" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="B28" s="21"/>
-      <c r="C28" s="29" t="s">
-        <v>27</v>
-      </c>
-      <c r="D28" s="30"/>
-      <c r="E28" s="22" t="s">
-        <v>28</v>
-      </c>
-      <c r="F28" s="23">
-        <v>0.6875</v>
-      </c>
-      <c r="G28" s="23">
-        <v>0.75</v>
-      </c>
-      <c r="H28" s="24"/>
-      <c r="I28" s="24"/>
-      <c r="J28" s="24"/>
-      <c r="K28" s="24">
-        <v>1.5</v>
-      </c>
-      <c r="L28" s="24"/>
-      <c r="M28" s="24"/>
-      <c r="N28" s="24"/>
-      <c r="O28" s="25"/>
-      <c r="P28" s="21"/>
-    </row>
-    <row r="29" spans="2:16" s="20" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="B29" s="21"/>
-      <c r="C29" s="29" t="s">
-        <v>27</v>
-      </c>
-      <c r="D29" s="30"/>
-      <c r="E29" s="22" t="s">
-        <v>28</v>
-      </c>
-      <c r="F29" s="23">
-        <v>0.6875</v>
-      </c>
-      <c r="G29" s="23">
-        <v>0.29166666666666669</v>
-      </c>
-      <c r="H29" s="24"/>
-      <c r="I29" s="24"/>
-      <c r="J29" s="24"/>
-      <c r="K29" s="24">
-        <v>0.5</v>
-      </c>
-      <c r="L29" s="24"/>
-      <c r="M29" s="24"/>
-      <c r="N29" s="24"/>
-      <c r="O29" s="25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="2:16" s="47" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="B28" s="48"/>
+      <c r="C28" s="67"/>
+      <c r="D28" s="68"/>
+      <c r="E28" s="49"/>
+      <c r="F28" s="50"/>
+      <c r="G28" s="50"/>
+      <c r="H28" s="51"/>
+      <c r="I28" s="51"/>
+      <c r="J28" s="51"/>
+      <c r="K28" s="51"/>
+      <c r="L28" s="51"/>
+      <c r="M28" s="51"/>
+      <c r="N28" s="51"/>
+      <c r="O28" s="84"/>
+      <c r="P28" s="48"/>
+    </row>
+    <row r="29" spans="2:16" s="47" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="B29" s="48"/>
+      <c r="C29" s="67"/>
+      <c r="D29" s="68"/>
+      <c r="E29" s="49"/>
+      <c r="F29" s="50"/>
+      <c r="G29" s="50"/>
+      <c r="H29" s="51"/>
+      <c r="I29" s="51"/>
+      <c r="J29" s="51"/>
+      <c r="K29" s="51"/>
+      <c r="L29" s="51"/>
+      <c r="M29" s="51"/>
+      <c r="N29" s="51"/>
+      <c r="O29" s="84">
         <f t="shared" si="0"/>
-        <v>0.5</v>
-      </c>
-      <c r="P29" s="21"/>
+        <v>0</v>
+      </c>
+      <c r="P29" s="48"/>
     </row>
     <row r="30" spans="2:16" x14ac:dyDescent="0.3">
-      <c r="C30" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="D30" s="28"/>
-      <c r="E30" s="12" t="s">
-        <v>28</v>
-      </c>
-      <c r="F30" s="13">
-        <v>0.25</v>
-      </c>
-      <c r="G30" s="13">
-        <v>0.29166666666666669</v>
-      </c>
+      <c r="C30" s="65"/>
+      <c r="D30" s="66"/>
+      <c r="E30" s="12"/>
+      <c r="F30" s="13"/>
+      <c r="G30" s="13"/>
       <c r="H30" s="14"/>
       <c r="I30" s="14"/>
       <c r="J30" s="14"/>
       <c r="K30" s="14"/>
-      <c r="L30" s="14">
-        <v>1</v>
-      </c>
+      <c r="L30" s="14"/>
       <c r="M30" s="14"/>
       <c r="N30" s="14"/>
-      <c r="O30" s="15">
+      <c r="O30" s="84">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="31" spans="2:16" x14ac:dyDescent="0.3">
-      <c r="C31" s="27" t="s">
-        <v>29</v>
-      </c>
-      <c r="D31" s="28"/>
-      <c r="E31" s="12" t="s">
-        <v>30</v>
-      </c>
-      <c r="F31" s="13">
-        <v>0.25</v>
-      </c>
-      <c r="G31" s="13">
-        <v>0.29166666666666669</v>
-      </c>
+      <c r="C31" s="65"/>
+      <c r="D31" s="66"/>
+      <c r="E31" s="12"/>
+      <c r="F31" s="13"/>
+      <c r="G31" s="13"/>
       <c r="H31" s="14"/>
       <c r="I31" s="14"/>
       <c r="J31" s="14"/>
       <c r="K31" s="14"/>
-      <c r="L31" s="14">
-        <v>1</v>
-      </c>
+      <c r="L31" s="14"/>
       <c r="M31" s="14"/>
       <c r="N31" s="14"/>
-      <c r="O31" s="15">
+      <c r="O31" s="84">
         <f>+SUM(H31:N31)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="32" spans="2:16" x14ac:dyDescent="0.3">
-      <c r="C32" s="27"/>
-      <c r="D32" s="28"/>
+      <c r="C32" s="65"/>
+      <c r="D32" s="66"/>
       <c r="E32" s="12"/>
       <c r="F32" s="13"/>
       <c r="G32" s="13"/>
@@ -1827,15 +2211,15 @@
       <c r="K32" s="14"/>
       <c r="L32" s="14"/>
       <c r="M32" s="14"/>
-      <c r="N32" s="16"/>
-      <c r="O32" s="15">
+      <c r="N32" s="15"/>
+      <c r="O32" s="84">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="3:18" x14ac:dyDescent="0.3">
-      <c r="C33" s="27"/>
-      <c r="D33" s="28"/>
+    <row r="33" spans="3:15" x14ac:dyDescent="0.3">
+      <c r="C33" s="65"/>
+      <c r="D33" s="66"/>
       <c r="E33" s="12"/>
       <c r="F33" s="13"/>
       <c r="G33" s="13"/>
@@ -1845,73 +2229,533 @@
       <c r="K33" s="14"/>
       <c r="L33" s="14"/>
       <c r="M33" s="14"/>
-      <c r="N33" s="16"/>
-      <c r="O33" s="15">
+      <c r="N33" s="15"/>
+      <c r="O33" s="84">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="3:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="C34" s="31"/>
-      <c r="D34" s="32"/>
+    <row r="34" spans="3:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="C34" s="69"/>
+      <c r="D34" s="70"/>
       <c r="E34" s="12"/>
       <c r="F34" s="13"/>
       <c r="G34" s="13"/>
-      <c r="H34" s="17">
+      <c r="H34" s="86">
         <f t="shared" ref="H34:N34" si="1">SUM(H26:H33)</f>
         <v>0</v>
       </c>
-      <c r="I34" s="17">
+      <c r="I34" s="86">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="J34" s="17">
+      <c r="J34" s="86">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="K34" s="17">
-        <f t="shared" si="1"/>
-        <v>4</v>
-      </c>
-      <c r="L34" s="17">
-        <f t="shared" si="1"/>
-        <v>2</v>
-      </c>
-      <c r="M34" s="17">
+      <c r="K34" s="86">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="N34" s="17">
+      <c r="L34" s="86">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="O34" s="18">
+      <c r="M34" s="86">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="N34" s="86">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="O34" s="85">
         <f>+SUM(H34:N34)</f>
-        <v>6</v>
-      </c>
-    </row>
-    <row r="35" spans="3:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="3:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C35" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="E35" s="19">
-        <v>3</v>
-      </c>
+      <c r="E35" s="16"/>
       <c r="F35" s="13"/>
       <c r="G35" s="13"/>
     </row>
-    <row r="36" spans="3:18" x14ac:dyDescent="0.3">
-      <c r="R36" t="s">
+    <row r="36" spans="3:15" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="E36" s="1"/>
+      <c r="G36" s="1"/>
+      <c r="H36" s="1"/>
+      <c r="I36" s="1"/>
+      <c r="J36" s="1"/>
+      <c r="K36" s="1"/>
+      <c r="L36" s="1"/>
+      <c r="M36" s="1"/>
+      <c r="N36" s="1"/>
+      <c r="O36" s="1"/>
+    </row>
+    <row r="37" spans="3:15" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="C37" s="56" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="37" spans="3:18" x14ac:dyDescent="0.3">
-      <c r="R37" s="4" t="s">
+      <c r="D37" s="56"/>
+      <c r="E37" s="56"/>
+      <c r="F37" s="56"/>
+      <c r="G37" s="56"/>
+      <c r="H37" s="56"/>
+      <c r="I37" s="56"/>
+      <c r="J37" s="56"/>
+      <c r="K37" s="56"/>
+      <c r="L37" s="56"/>
+      <c r="M37" s="56"/>
+      <c r="N37" s="56"/>
+      <c r="O37" s="56"/>
+    </row>
+    <row r="38" spans="3:15" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="C38" s="56"/>
+      <c r="D38" s="56"/>
+      <c r="E38" s="56"/>
+      <c r="F38" s="56"/>
+      <c r="G38" s="56"/>
+      <c r="H38" s="56"/>
+      <c r="I38" s="56"/>
+      <c r="J38" s="56"/>
+      <c r="K38" s="56"/>
+      <c r="L38" s="56"/>
+      <c r="M38" s="56"/>
+      <c r="N38" s="56"/>
+      <c r="O38" s="56"/>
+    </row>
+    <row r="39" spans="3:15" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="G39" s="1"/>
+      <c r="H39" s="1"/>
+      <c r="I39" s="1"/>
+      <c r="J39" s="1"/>
+      <c r="K39" s="1"/>
+      <c r="L39" s="1"/>
+      <c r="M39" s="1"/>
+      <c r="N39" s="1"/>
+      <c r="O39" s="1"/>
+    </row>
+    <row r="40" spans="3:15" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="C40" s="17"/>
+      <c r="D40" s="17"/>
+      <c r="E40" s="17"/>
+      <c r="F40" s="17"/>
+      <c r="G40" s="18"/>
+      <c r="H40" s="18"/>
+      <c r="I40" s="18"/>
+      <c r="J40" s="18"/>
+      <c r="K40" s="18"/>
+      <c r="L40" s="18"/>
+      <c r="M40" s="18"/>
+      <c r="N40" s="18"/>
+      <c r="O40" s="18"/>
+    </row>
+    <row r="41" spans="3:15" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="C41" s="19"/>
+      <c r="D41" s="19"/>
+      <c r="E41" s="19"/>
+      <c r="F41" s="19"/>
+      <c r="G41" s="20"/>
+      <c r="H41" s="20"/>
+      <c r="I41" s="20"/>
+      <c r="J41" s="20"/>
+      <c r="K41" s="20"/>
+      <c r="L41" s="20"/>
+      <c r="M41" s="20"/>
+      <c r="N41" s="20"/>
+      <c r="O41" s="20"/>
+    </row>
+    <row r="42" spans="3:15" customFormat="1" ht="23.4" x14ac:dyDescent="0.45">
+      <c r="C42" s="71" t="s">
         <v>20</v>
       </c>
+      <c r="D42" s="72"/>
+      <c r="E42" s="72"/>
+      <c r="F42" s="72"/>
+      <c r="G42" s="72"/>
+      <c r="H42" s="72"/>
+      <c r="I42" s="72"/>
+      <c r="J42" s="72"/>
+      <c r="K42" s="72"/>
+      <c r="L42" s="72"/>
+      <c r="M42" s="72"/>
+      <c r="N42" s="72"/>
+      <c r="O42" s="73"/>
+    </row>
+    <row r="43" spans="3:15" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="C43" s="61" t="s">
+        <v>4</v>
+      </c>
+      <c r="D43" s="62"/>
+      <c r="E43" s="74"/>
+      <c r="F43" s="74"/>
+      <c r="G43" s="74"/>
+      <c r="H43" s="74"/>
+      <c r="I43" s="74"/>
+      <c r="J43" s="74"/>
+      <c r="K43" s="74"/>
+      <c r="L43" s="74"/>
+      <c r="M43" s="74"/>
+      <c r="N43" s="74"/>
+      <c r="O43" s="74"/>
+    </row>
+    <row r="44" spans="3:15" x14ac:dyDescent="0.3">
+      <c r="C44" s="61" t="s">
+        <v>21</v>
+      </c>
+      <c r="D44" s="62"/>
+      <c r="E44" s="63"/>
+      <c r="F44" s="63"/>
+      <c r="G44" s="63"/>
+      <c r="O44" s="21"/>
+    </row>
+    <row r="45" spans="3:15" x14ac:dyDescent="0.3">
+      <c r="C45" s="61" t="s">
+        <v>22</v>
+      </c>
+      <c r="D45" s="62"/>
+      <c r="E45" s="63"/>
+      <c r="F45" s="63"/>
+      <c r="G45" s="63"/>
+      <c r="O45" s="21"/>
+    </row>
+    <row r="46" spans="3:15" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="C46" s="61" t="s">
+        <v>23</v>
+      </c>
+      <c r="D46" s="62"/>
+      <c r="E46" s="64"/>
+      <c r="F46" s="64"/>
+      <c r="G46" s="64"/>
+      <c r="H46" s="64"/>
+      <c r="I46" s="64"/>
+      <c r="J46" s="64"/>
+      <c r="K46" s="64"/>
+      <c r="L46" s="64"/>
+      <c r="M46" s="64"/>
+      <c r="N46" s="64"/>
+      <c r="O46" s="64"/>
+    </row>
+    <row r="47" spans="3:15" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="C47" s="61" t="s">
+        <v>24</v>
+      </c>
+      <c r="D47" s="62"/>
+      <c r="E47" s="64"/>
+      <c r="F47" s="64"/>
+      <c r="G47" s="64"/>
+      <c r="H47" s="64"/>
+      <c r="I47" s="64"/>
+      <c r="J47" s="64"/>
+      <c r="K47" s="64"/>
+      <c r="L47" s="64"/>
+      <c r="M47" s="64"/>
+      <c r="N47" s="64"/>
+      <c r="O47" s="64"/>
+    </row>
+    <row r="48" spans="3:15" x14ac:dyDescent="0.3">
+      <c r="C48" s="22" t="s">
+        <v>25</v>
+      </c>
+      <c r="D48" s="23"/>
+      <c r="H48" s="24" t="s">
+        <v>35</v>
+      </c>
+      <c r="O48" s="21"/>
+    </row>
+    <row r="49" spans="3:18" x14ac:dyDescent="0.3">
+      <c r="C49" s="22" t="s">
+        <v>26</v>
+      </c>
+      <c r="D49" s="23"/>
+      <c r="F49" s="24" t="s">
+        <v>35</v>
+      </c>
+      <c r="O49" s="21"/>
+    </row>
+    <row r="50" spans="3:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="C50" s="22"/>
+      <c r="D50" s="23"/>
+      <c r="O50" s="21"/>
+    </row>
+    <row r="51" spans="3:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="C51" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="D51" s="23"/>
+      <c r="E51" s="25"/>
+      <c r="F51" s="25" t="s">
+        <v>28</v>
+      </c>
+      <c r="G51" s="26"/>
+      <c r="H51" s="25"/>
+      <c r="I51" s="25"/>
+      <c r="J51" s="25" t="s">
+        <v>29</v>
+      </c>
+      <c r="K51" s="27"/>
+      <c r="L51" s="25" t="s">
+        <v>30</v>
+      </c>
+      <c r="M51" s="28"/>
+      <c r="O51" s="21"/>
+      <c r="R51" s="5" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="52" spans="3:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="C52" s="29" t="s">
+        <v>32</v>
+      </c>
+      <c r="D52"/>
+      <c r="E52" s="25"/>
+      <c r="F52" s="25" t="s">
+        <v>33</v>
+      </c>
+      <c r="G52" s="26"/>
+      <c r="H52" s="25"/>
+      <c r="I52" s="25"/>
+      <c r="J52" s="25" t="s">
+        <v>34</v>
+      </c>
+      <c r="K52" s="27"/>
+      <c r="L52" s="25" t="s">
+        <v>30</v>
+      </c>
+      <c r="M52" s="30"/>
+      <c r="O52" s="21"/>
+      <c r="R52" s="5" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="53" spans="3:18" x14ac:dyDescent="0.3">
+      <c r="C53" s="29"/>
+      <c r="D53"/>
+      <c r="E53" s="25"/>
+      <c r="F53" s="25"/>
+      <c r="G53" s="25"/>
+      <c r="H53" s="25"/>
+      <c r="I53" s="25"/>
+      <c r="K53" s="25"/>
+      <c r="M53" s="25"/>
+      <c r="N53" s="25"/>
+      <c r="O53" s="31"/>
+    </row>
+    <row r="54" spans="3:18" x14ac:dyDescent="0.3">
+      <c r="C54" s="22" t="s">
+        <v>36</v>
+      </c>
+      <c r="D54"/>
+      <c r="E54"/>
+      <c r="F54"/>
+      <c r="G54" s="1"/>
+      <c r="H54" s="1"/>
+      <c r="I54" s="1"/>
+      <c r="J54" s="1"/>
+      <c r="K54" s="1"/>
+      <c r="L54" s="1"/>
+      <c r="M54" s="1"/>
+      <c r="N54" s="1"/>
+      <c r="O54" s="32"/>
+    </row>
+    <row r="55" spans="3:18" x14ac:dyDescent="0.3">
+      <c r="C55" s="33"/>
+      <c r="D55" s="34"/>
+      <c r="E55" s="34"/>
+      <c r="F55" s="34"/>
+      <c r="G55" s="35"/>
+      <c r="H55" s="35"/>
+      <c r="I55" s="35"/>
+      <c r="J55" s="35"/>
+      <c r="K55" s="35"/>
+      <c r="L55" s="35"/>
+      <c r="M55" s="35"/>
+      <c r="N55" s="35"/>
+      <c r="O55" s="36"/>
+    </row>
+    <row r="56" spans="3:18" x14ac:dyDescent="0.3">
+      <c r="C56" s="37"/>
+      <c r="D56" s="38"/>
+      <c r="E56" s="38"/>
+      <c r="F56" s="38"/>
+      <c r="G56" s="39"/>
+      <c r="H56" s="39"/>
+      <c r="I56" s="39"/>
+      <c r="J56" s="39"/>
+      <c r="K56" s="39"/>
+      <c r="L56" s="39"/>
+      <c r="M56" s="39"/>
+      <c r="N56" s="39"/>
+      <c r="O56" s="40"/>
+    </row>
+    <row r="57" spans="3:18" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="C57" s="29"/>
+      <c r="E57" s="41"/>
+      <c r="F57" s="41"/>
+      <c r="G57" s="42"/>
+      <c r="H57" s="42"/>
+      <c r="I57" s="42"/>
+      <c r="J57" s="42"/>
+      <c r="K57" s="1"/>
+      <c r="L57" s="1"/>
+      <c r="M57" s="1"/>
+      <c r="N57" s="1"/>
+      <c r="O57" s="32"/>
+    </row>
+    <row r="58" spans="3:18" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="C58" s="29"/>
+      <c r="G58" s="1"/>
+      <c r="H58" s="1"/>
+      <c r="I58" s="1"/>
+      <c r="J58" s="1"/>
+      <c r="K58" s="1"/>
+      <c r="L58" s="1"/>
+      <c r="M58" s="1"/>
+      <c r="N58" s="1"/>
+      <c r="O58" s="32"/>
+    </row>
+    <row r="59" spans="3:18" x14ac:dyDescent="0.3">
+      <c r="C59" s="29" t="s">
+        <v>37</v>
+      </c>
+      <c r="D59"/>
+      <c r="E59" s="52"/>
+      <c r="F59" s="52"/>
+      <c r="G59" s="52"/>
+      <c r="H59" s="52"/>
+      <c r="I59" s="52"/>
+      <c r="J59" s="52"/>
+      <c r="O59" s="21"/>
+    </row>
+    <row r="60" spans="3:18" x14ac:dyDescent="0.3">
+      <c r="C60" s="29" t="s">
+        <v>38</v>
+      </c>
+      <c r="D60"/>
+      <c r="E60" s="52" t="s">
+        <v>39</v>
+      </c>
+      <c r="F60" s="52"/>
+      <c r="G60" s="52"/>
+      <c r="H60" s="52"/>
+      <c r="I60" s="52"/>
+      <c r="J60" s="52"/>
+      <c r="O60" s="21"/>
+    </row>
+    <row r="61" spans="3:18" ht="35.1" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C61" s="53" t="s">
+        <v>40</v>
+      </c>
+      <c r="D61" s="54"/>
+      <c r="E61" s="52"/>
+      <c r="F61" s="52"/>
+      <c r="O61" s="21"/>
+      <c r="R61" s="4" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="62" spans="3:18" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="C62" s="43"/>
+      <c r="D62" s="44"/>
+      <c r="E62" s="44"/>
+      <c r="F62" s="44"/>
+      <c r="G62" s="45"/>
+      <c r="H62" s="45"/>
+      <c r="I62" s="45"/>
+      <c r="J62" s="45"/>
+      <c r="K62" s="45"/>
+      <c r="L62" s="45"/>
+      <c r="M62" s="45"/>
+      <c r="N62" s="45"/>
+      <c r="O62" s="46"/>
+      <c r="R62" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="63" spans="3:18" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="C63" s="55" t="s">
+        <v>42</v>
+      </c>
+      <c r="D63" s="56"/>
+      <c r="E63" s="56"/>
+      <c r="F63" s="56"/>
+      <c r="G63" s="56"/>
+      <c r="H63" s="56"/>
+      <c r="I63" s="56"/>
+      <c r="J63" s="56"/>
+      <c r="K63" s="56"/>
+      <c r="L63" s="56"/>
+      <c r="M63" s="56"/>
+      <c r="N63" s="56"/>
+      <c r="O63" s="57"/>
+      <c r="R63" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="64" spans="3:18" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="C64" s="55"/>
+      <c r="D64" s="56"/>
+      <c r="E64" s="56"/>
+      <c r="F64" s="56"/>
+      <c r="G64" s="56"/>
+      <c r="H64" s="56"/>
+      <c r="I64" s="56"/>
+      <c r="J64" s="56"/>
+      <c r="K64" s="56"/>
+      <c r="L64" s="56"/>
+      <c r="M64" s="56"/>
+      <c r="N64" s="56"/>
+      <c r="O64" s="57"/>
+      <c r="R64" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="65" spans="3:18" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="C65" s="58"/>
+      <c r="D65" s="59"/>
+      <c r="E65" s="59"/>
+      <c r="F65" s="59"/>
+      <c r="G65" s="59"/>
+      <c r="H65" s="59"/>
+      <c r="I65" s="59"/>
+      <c r="J65" s="59"/>
+      <c r="K65" s="59"/>
+      <c r="L65" s="59"/>
+      <c r="M65" s="59"/>
+      <c r="N65" s="59"/>
+      <c r="O65" s="60"/>
+      <c r="R65" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="66" spans="3:18" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="G66" s="1"/>
+      <c r="H66" s="1"/>
+      <c r="I66" s="1"/>
+      <c r="J66" s="1"/>
+      <c r="K66" s="1"/>
+      <c r="L66" s="1"/>
+      <c r="M66" s="1"/>
+      <c r="N66" s="1"/>
+      <c r="O66" s="1"/>
+      <c r="R66" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="67" spans="3:18" x14ac:dyDescent="0.3">
+      <c r="R67" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="68" spans="3:18" x14ac:dyDescent="0.3">
+      <c r="R68" s="4" t="s">
+        <v>48</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="23">
+  <mergeCells count="40">
     <mergeCell ref="C11:O11"/>
     <mergeCell ref="C14:D14"/>
     <mergeCell ref="E14:O14"/>
@@ -1927,6 +2771,8 @@
     <mergeCell ref="C18:D19"/>
     <mergeCell ref="E19:O19"/>
     <mergeCell ref="E20:O20"/>
+    <mergeCell ref="C44:D44"/>
+    <mergeCell ref="E44:G44"/>
     <mergeCell ref="C27:D27"/>
     <mergeCell ref="C29:D29"/>
     <mergeCell ref="C30:D30"/>
@@ -1934,8 +2780,31 @@
     <mergeCell ref="C32:D32"/>
     <mergeCell ref="C33:D33"/>
     <mergeCell ref="C34:D34"/>
+    <mergeCell ref="C37:O38"/>
+    <mergeCell ref="C42:O42"/>
+    <mergeCell ref="C43:D43"/>
+    <mergeCell ref="E43:O43"/>
     <mergeCell ref="C28:D28"/>
+    <mergeCell ref="C45:D45"/>
+    <mergeCell ref="E45:G45"/>
+    <mergeCell ref="C46:D46"/>
+    <mergeCell ref="E46:O46"/>
+    <mergeCell ref="C47:D47"/>
+    <mergeCell ref="E47:O47"/>
+    <mergeCell ref="E59:J59"/>
+    <mergeCell ref="E60:J60"/>
+    <mergeCell ref="C61:D61"/>
+    <mergeCell ref="E61:F61"/>
+    <mergeCell ref="C63:O65"/>
   </mergeCells>
+  <dataValidations count="2">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E60:J60" xr:uid="{EED16A01-C090-44A9-A7D6-FC173323C962}">
+      <formula1>$R$61:$R$68</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F49:F50 H48" xr:uid="{E8977EEB-19F9-4AF2-8C47-26A586CFF158}">
+      <formula1>$R$49:$R$52</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
   <legacyDrawing r:id="rId2"/>
@@ -1950,14 +2819,14 @@
                   <from>
                     <xdr:col>6</xdr:col>
                     <xdr:colOff>289560</xdr:colOff>
-                    <xdr:row>35</xdr:row>
-                    <xdr:rowOff>0</xdr:rowOff>
+                    <xdr:row>49</xdr:row>
+                    <xdr:rowOff>182880</xdr:rowOff>
                   </from>
                   <to>
                     <xdr:col>6</xdr:col>
                     <xdr:colOff>533400</xdr:colOff>
-                    <xdr:row>36</xdr:row>
-                    <xdr:rowOff>53340</xdr:rowOff>
+                    <xdr:row>51</xdr:row>
+                    <xdr:rowOff>38100</xdr:rowOff>
                   </to>
                 </anchor>
               </controlPr>
@@ -1972,14 +2841,14 @@
                   <from>
                     <xdr:col>6</xdr:col>
                     <xdr:colOff>289560</xdr:colOff>
-                    <xdr:row>35</xdr:row>
-                    <xdr:rowOff>0</xdr:rowOff>
+                    <xdr:row>50</xdr:row>
+                    <xdr:rowOff>190500</xdr:rowOff>
                   </from>
                   <to>
                     <xdr:col>6</xdr:col>
                     <xdr:colOff>533400</xdr:colOff>
-                    <xdr:row>36</xdr:row>
-                    <xdr:rowOff>53340</xdr:rowOff>
+                    <xdr:row>52</xdr:row>
+                    <xdr:rowOff>45720</xdr:rowOff>
                   </to>
                 </anchor>
               </controlPr>
@@ -1994,14 +2863,14 @@
                   <from>
                     <xdr:col>10</xdr:col>
                     <xdr:colOff>251460</xdr:colOff>
-                    <xdr:row>35</xdr:row>
-                    <xdr:rowOff>0</xdr:rowOff>
+                    <xdr:row>49</xdr:row>
+                    <xdr:rowOff>190500</xdr:rowOff>
                   </from>
                   <to>
                     <xdr:col>10</xdr:col>
                     <xdr:colOff>495300</xdr:colOff>
-                    <xdr:row>36</xdr:row>
-                    <xdr:rowOff>45720</xdr:rowOff>
+                    <xdr:row>51</xdr:row>
+                    <xdr:rowOff>38100</xdr:rowOff>
                   </to>
                 </anchor>
               </controlPr>
@@ -2016,14 +2885,14 @@
                   <from>
                     <xdr:col>10</xdr:col>
                     <xdr:colOff>251460</xdr:colOff>
-                    <xdr:row>35</xdr:row>
+                    <xdr:row>51</xdr:row>
                     <xdr:rowOff>0</xdr:rowOff>
                   </from>
                   <to>
                     <xdr:col>10</xdr:col>
                     <xdr:colOff>495300</xdr:colOff>
-                    <xdr:row>36</xdr:row>
-                    <xdr:rowOff>45720</xdr:rowOff>
+                    <xdr:row>52</xdr:row>
+                    <xdr:rowOff>38100</xdr:rowOff>
                   </to>
                 </anchor>
               </controlPr>

</xml_diff>

<commit_message>
Actualizar plantilla de horas extras con formulas
</commit_message>
<xml_diff>
--- a/public/plantilla-horas-extra.xlsx
+++ b/public/plantilla-horas-extra.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\proyecto\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{CCE3ABAA-C510-42C1-A3C3-33A08F2CD770}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{4ED5E154-E3DB-41F2-B66F-76C0C4C3461A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{44F16EB2-3180-4466-BB78-D60D707A8425}"/>
   </bookViews>
@@ -937,6 +937,98 @@
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="166" fontId="0" fillId="4" borderId="15" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="4" borderId="20" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="4" borderId="19" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
       <protection locked="0"/>
@@ -950,9 +1042,6 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
@@ -964,95 +1053,6 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="4" borderId="15" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="4" borderId="20" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="4" borderId="19" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1831,21 +1831,21 @@
       <c r="O10" s="1"/>
     </row>
     <row r="11" spans="3:16" customFormat="1" ht="29.4" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="C11" s="80" t="s">
+      <c r="C11" s="55" t="s">
         <v>0</v>
       </c>
-      <c r="D11" s="81"/>
-      <c r="E11" s="81"/>
-      <c r="F11" s="81"/>
-      <c r="G11" s="81"/>
-      <c r="H11" s="81"/>
-      <c r="I11" s="81"/>
-      <c r="J11" s="81"/>
-      <c r="K11" s="81"/>
-      <c r="L11" s="81"/>
-      <c r="M11" s="81"/>
-      <c r="N11" s="81"/>
-      <c r="O11" s="82"/>
+      <c r="D11" s="56"/>
+      <c r="E11" s="56"/>
+      <c r="F11" s="56"/>
+      <c r="G11" s="56"/>
+      <c r="H11" s="56"/>
+      <c r="I11" s="56"/>
+      <c r="J11" s="56"/>
+      <c r="K11" s="56"/>
+      <c r="L11" s="56"/>
+      <c r="M11" s="56"/>
+      <c r="N11" s="56"/>
+      <c r="O11" s="57"/>
     </row>
     <row r="12" spans="3:16" customFormat="1" ht="15.9" customHeight="1" x14ac:dyDescent="0.4">
       <c r="C12" s="3"/>
@@ -1878,108 +1878,108 @@
       <c r="O13" s="3"/>
     </row>
     <row r="14" spans="3:16" ht="15.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C14" s="75" t="s">
+      <c r="C14" s="58" t="s">
         <v>1</v>
       </c>
-      <c r="D14" s="75"/>
-      <c r="E14" s="83"/>
-      <c r="F14" s="83"/>
-      <c r="G14" s="83"/>
-      <c r="H14" s="83"/>
-      <c r="I14" s="83"/>
-      <c r="J14" s="83"/>
-      <c r="K14" s="83"/>
-      <c r="L14" s="83"/>
-      <c r="M14" s="83"/>
-      <c r="N14" s="83"/>
-      <c r="O14" s="83"/>
+      <c r="D14" s="58"/>
+      <c r="E14" s="59"/>
+      <c r="F14" s="59"/>
+      <c r="G14" s="59"/>
+      <c r="H14" s="59"/>
+      <c r="I14" s="59"/>
+      <c r="J14" s="59"/>
+      <c r="K14" s="59"/>
+      <c r="L14" s="59"/>
+      <c r="M14" s="59"/>
+      <c r="N14" s="59"/>
+      <c r="O14" s="59"/>
     </row>
     <row r="15" spans="3:16" ht="15.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C15" s="75" t="s">
+      <c r="C15" s="58" t="s">
         <v>2</v>
       </c>
-      <c r="D15" s="75"/>
-      <c r="E15" s="64"/>
-      <c r="F15" s="64"/>
-      <c r="G15" s="64"/>
-      <c r="H15" s="64"/>
-      <c r="I15" s="64"/>
-      <c r="J15" s="64"/>
-      <c r="K15" s="64"/>
-      <c r="L15" s="64"/>
-      <c r="M15" s="64"/>
-      <c r="N15" s="64"/>
-      <c r="O15" s="64"/>
+      <c r="D15" s="58"/>
+      <c r="E15" s="60"/>
+      <c r="F15" s="60"/>
+      <c r="G15" s="60"/>
+      <c r="H15" s="60"/>
+      <c r="I15" s="60"/>
+      <c r="J15" s="60"/>
+      <c r="K15" s="60"/>
+      <c r="L15" s="60"/>
+      <c r="M15" s="60"/>
+      <c r="N15" s="60"/>
+      <c r="O15" s="60"/>
     </row>
     <row r="16" spans="3:16" ht="15.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C16" s="75" t="s">
+      <c r="C16" s="58" t="s">
         <v>3</v>
       </c>
-      <c r="D16" s="75"/>
-      <c r="E16" s="74"/>
-      <c r="F16" s="74"/>
-      <c r="G16" s="74"/>
-      <c r="H16" s="74"/>
-      <c r="I16" s="74"/>
-      <c r="J16" s="74"/>
-      <c r="K16" s="74"/>
-      <c r="L16" s="74"/>
-      <c r="M16" s="74"/>
-      <c r="N16" s="74"/>
-      <c r="O16" s="74"/>
+      <c r="D16" s="58"/>
+      <c r="E16" s="66"/>
+      <c r="F16" s="66"/>
+      <c r="G16" s="66"/>
+      <c r="H16" s="66"/>
+      <c r="I16" s="66"/>
+      <c r="J16" s="66"/>
+      <c r="K16" s="66"/>
+      <c r="L16" s="66"/>
+      <c r="M16" s="66"/>
+      <c r="N16" s="66"/>
+      <c r="O16" s="66"/>
     </row>
     <row r="17" spans="2:16" ht="15.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C17" s="75" t="s">
+      <c r="C17" s="58" t="s">
         <v>4</v>
       </c>
-      <c r="D17" s="75"/>
-      <c r="E17" s="74"/>
-      <c r="F17" s="74"/>
-      <c r="G17" s="74"/>
-      <c r="H17" s="74"/>
-      <c r="I17" s="74"/>
-      <c r="J17" s="74"/>
-      <c r="K17" s="74"/>
-      <c r="L17" s="74"/>
-      <c r="M17" s="74"/>
-      <c r="N17" s="74"/>
-      <c r="O17" s="74"/>
+      <c r="D17" s="58"/>
+      <c r="E17" s="66"/>
+      <c r="F17" s="66"/>
+      <c r="G17" s="66"/>
+      <c r="H17" s="66"/>
+      <c r="I17" s="66"/>
+      <c r="J17" s="66"/>
+      <c r="K17" s="66"/>
+      <c r="L17" s="66"/>
+      <c r="M17" s="66"/>
+      <c r="N17" s="66"/>
+      <c r="O17" s="66"/>
     </row>
     <row r="18" spans="2:16" ht="15.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C18" s="76" t="s">
+      <c r="C18" s="67" t="s">
         <v>5</v>
       </c>
-      <c r="D18" s="76"/>
+      <c r="D18" s="67"/>
     </row>
     <row r="19" spans="2:16" ht="15.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C19" s="76"/>
-      <c r="D19" s="76"/>
-      <c r="E19" s="74"/>
-      <c r="F19" s="74"/>
-      <c r="G19" s="74"/>
-      <c r="H19" s="74"/>
-      <c r="I19" s="74"/>
-      <c r="J19" s="74"/>
-      <c r="K19" s="74"/>
-      <c r="L19" s="74"/>
-      <c r="M19" s="74"/>
-      <c r="N19" s="74"/>
-      <c r="O19" s="74"/>
+      <c r="C19" s="67"/>
+      <c r="D19" s="67"/>
+      <c r="E19" s="66"/>
+      <c r="F19" s="66"/>
+      <c r="G19" s="66"/>
+      <c r="H19" s="66"/>
+      <c r="I19" s="66"/>
+      <c r="J19" s="66"/>
+      <c r="K19" s="66"/>
+      <c r="L19" s="66"/>
+      <c r="M19" s="66"/>
+      <c r="N19" s="66"/>
+      <c r="O19" s="66"/>
     </row>
     <row r="20" spans="2:16" ht="15.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C20"/>
       <c r="D20"/>
-      <c r="E20" s="74"/>
-      <c r="F20" s="74"/>
-      <c r="G20" s="74"/>
-      <c r="H20" s="74"/>
-      <c r="I20" s="74"/>
-      <c r="J20" s="74"/>
-      <c r="K20" s="74"/>
-      <c r="L20" s="74"/>
-      <c r="M20" s="74"/>
-      <c r="N20" s="74"/>
-      <c r="O20" s="74"/>
+      <c r="E20" s="66"/>
+      <c r="F20" s="66"/>
+      <c r="G20" s="66"/>
+      <c r="H20" s="66"/>
+      <c r="I20" s="66"/>
+      <c r="J20" s="66"/>
+      <c r="K20" s="66"/>
+      <c r="L20" s="66"/>
+      <c r="M20" s="66"/>
+      <c r="N20" s="66"/>
+      <c r="O20" s="66"/>
     </row>
     <row r="21" spans="2:16" customFormat="1" ht="15.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="G21" s="1"/>
@@ -1993,36 +1993,36 @@
       <c r="O21" s="1"/>
     </row>
     <row r="22" spans="2:16" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="C22" s="77" t="s">
+      <c r="C22" s="61" t="s">
         <v>6</v>
       </c>
-      <c r="D22" s="77"/>
-      <c r="E22" s="77"/>
-      <c r="F22" s="77"/>
-      <c r="G22" s="77"/>
-      <c r="H22" s="77"/>
-      <c r="I22" s="77"/>
-      <c r="J22" s="77"/>
-      <c r="K22" s="77"/>
-      <c r="L22" s="77"/>
-      <c r="M22" s="77"/>
-      <c r="N22" s="77"/>
-      <c r="O22" s="77"/>
+      <c r="D22" s="61"/>
+      <c r="E22" s="61"/>
+      <c r="F22" s="61"/>
+      <c r="G22" s="61"/>
+      <c r="H22" s="61"/>
+      <c r="I22" s="61"/>
+      <c r="J22" s="61"/>
+      <c r="K22" s="61"/>
+      <c r="L22" s="61"/>
+      <c r="M22" s="61"/>
+      <c r="N22" s="61"/>
+      <c r="O22" s="61"/>
     </row>
     <row r="23" spans="2:16" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="C23" s="77"/>
-      <c r="D23" s="77"/>
-      <c r="E23" s="77"/>
-      <c r="F23" s="77"/>
-      <c r="G23" s="77"/>
-      <c r="H23" s="77"/>
-      <c r="I23" s="77"/>
-      <c r="J23" s="77"/>
-      <c r="K23" s="77"/>
-      <c r="L23" s="77"/>
-      <c r="M23" s="77"/>
-      <c r="N23" s="77"/>
-      <c r="O23" s="77"/>
+      <c r="C23" s="61"/>
+      <c r="D23" s="61"/>
+      <c r="E23" s="61"/>
+      <c r="F23" s="61"/>
+      <c r="G23" s="61"/>
+      <c r="H23" s="61"/>
+      <c r="I23" s="61"/>
+      <c r="J23" s="61"/>
+      <c r="K23" s="61"/>
+      <c r="L23" s="61"/>
+      <c r="M23" s="61"/>
+      <c r="N23" s="61"/>
+      <c r="O23" s="61"/>
     </row>
     <row r="24" spans="2:16" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="G24" s="1"/>
@@ -2050,10 +2050,10 @@
       <c r="O24" s="1"/>
     </row>
     <row r="25" spans="2:16" s="11" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="C25" s="78" t="s">
+      <c r="C25" s="62" t="s">
         <v>13</v>
       </c>
-      <c r="D25" s="79"/>
+      <c r="D25" s="63"/>
       <c r="E25" s="7" t="s">
         <v>14</v>
       </c>
@@ -2090,8 +2090,8 @@
     </row>
     <row r="26" spans="2:16" s="47" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B26" s="48"/>
-      <c r="C26" s="67"/>
-      <c r="D26" s="68"/>
+      <c r="C26" s="64"/>
+      <c r="D26" s="65"/>
       <c r="E26" s="49"/>
       <c r="F26" s="50"/>
       <c r="G26" s="50"/>
@@ -2102,15 +2102,15 @@
       <c r="L26" s="51"/>
       <c r="M26" s="51"/>
       <c r="N26" s="51"/>
-      <c r="O26" s="84">
+      <c r="O26" s="52">
         <f>+SUM(H26:N26)</f>
         <v>0</v>
       </c>
       <c r="P26" s="48"/>
     </row>
     <row r="27" spans="2:16" x14ac:dyDescent="0.3">
-      <c r="C27" s="65"/>
-      <c r="D27" s="66"/>
+      <c r="C27" s="71"/>
+      <c r="D27" s="72"/>
       <c r="E27" s="12"/>
       <c r="F27" s="13"/>
       <c r="G27" s="13"/>
@@ -2121,15 +2121,15 @@
       <c r="L27" s="14"/>
       <c r="M27" s="14"/>
       <c r="N27" s="14"/>
-      <c r="O27" s="84">
+      <c r="O27" s="52">
         <f t="shared" ref="O27:O33" si="0">+SUM(H27:N27)</f>
         <v>0</v>
       </c>
     </row>
     <row r="28" spans="2:16" s="47" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B28" s="48"/>
-      <c r="C28" s="67"/>
-      <c r="D28" s="68"/>
+      <c r="C28" s="64"/>
+      <c r="D28" s="65"/>
       <c r="E28" s="49"/>
       <c r="F28" s="50"/>
       <c r="G28" s="50"/>
@@ -2140,13 +2140,13 @@
       <c r="L28" s="51"/>
       <c r="M28" s="51"/>
       <c r="N28" s="51"/>
-      <c r="O28" s="84"/>
+      <c r="O28" s="52"/>
       <c r="P28" s="48"/>
     </row>
     <row r="29" spans="2:16" s="47" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B29" s="48"/>
-      <c r="C29" s="67"/>
-      <c r="D29" s="68"/>
+      <c r="C29" s="64"/>
+      <c r="D29" s="65"/>
       <c r="E29" s="49"/>
       <c r="F29" s="50"/>
       <c r="G29" s="50"/>
@@ -2157,15 +2157,15 @@
       <c r="L29" s="51"/>
       <c r="M29" s="51"/>
       <c r="N29" s="51"/>
-      <c r="O29" s="84">
+      <c r="O29" s="52">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="P29" s="48"/>
     </row>
     <row r="30" spans="2:16" x14ac:dyDescent="0.3">
-      <c r="C30" s="65"/>
-      <c r="D30" s="66"/>
+      <c r="C30" s="71"/>
+      <c r="D30" s="72"/>
       <c r="E30" s="12"/>
       <c r="F30" s="13"/>
       <c r="G30" s="13"/>
@@ -2176,14 +2176,14 @@
       <c r="L30" s="14"/>
       <c r="M30" s="14"/>
       <c r="N30" s="14"/>
-      <c r="O30" s="84">
+      <c r="O30" s="52">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
     <row r="31" spans="2:16" x14ac:dyDescent="0.3">
-      <c r="C31" s="65"/>
-      <c r="D31" s="66"/>
+      <c r="C31" s="71"/>
+      <c r="D31" s="72"/>
       <c r="E31" s="12"/>
       <c r="F31" s="13"/>
       <c r="G31" s="13"/>
@@ -2194,14 +2194,14 @@
       <c r="L31" s="14"/>
       <c r="M31" s="14"/>
       <c r="N31" s="14"/>
-      <c r="O31" s="84">
+      <c r="O31" s="52">
         <f>+SUM(H31:N31)</f>
         <v>0</v>
       </c>
     </row>
     <row r="32" spans="2:16" x14ac:dyDescent="0.3">
-      <c r="C32" s="65"/>
-      <c r="D32" s="66"/>
+      <c r="C32" s="71"/>
+      <c r="D32" s="72"/>
       <c r="E32" s="12"/>
       <c r="F32" s="13"/>
       <c r="G32" s="13"/>
@@ -2212,14 +2212,14 @@
       <c r="L32" s="14"/>
       <c r="M32" s="14"/>
       <c r="N32" s="15"/>
-      <c r="O32" s="84">
+      <c r="O32" s="52">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
     <row r="33" spans="3:15" x14ac:dyDescent="0.3">
-      <c r="C33" s="65"/>
-      <c r="D33" s="66"/>
+      <c r="C33" s="71"/>
+      <c r="D33" s="72"/>
       <c r="E33" s="12"/>
       <c r="F33" s="13"/>
       <c r="G33" s="13"/>
@@ -2230,46 +2230,46 @@
       <c r="L33" s="14"/>
       <c r="M33" s="14"/>
       <c r="N33" s="15"/>
-      <c r="O33" s="84">
+      <c r="O33" s="52">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
     <row r="34" spans="3:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="C34" s="69"/>
-      <c r="D34" s="70"/>
+      <c r="C34" s="73"/>
+      <c r="D34" s="74"/>
       <c r="E34" s="12"/>
       <c r="F34" s="13"/>
       <c r="G34" s="13"/>
-      <c r="H34" s="86">
+      <c r="H34" s="54">
         <f t="shared" ref="H34:N34" si="1">SUM(H26:H33)</f>
         <v>0</v>
       </c>
-      <c r="I34" s="86">
+      <c r="I34" s="54">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="J34" s="86">
+      <c r="J34" s="54">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="K34" s="86">
+      <c r="K34" s="54">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="L34" s="86">
+      <c r="L34" s="54">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="M34" s="86">
+      <c r="M34" s="54">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="N34" s="86">
+      <c r="N34" s="54">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="O34" s="85">
+      <c r="O34" s="53">
         <f>+SUM(H34:N34)</f>
         <v>0</v>
       </c>
@@ -2295,36 +2295,36 @@
       <c r="O36" s="1"/>
     </row>
     <row r="37" spans="3:15" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="C37" s="56" t="s">
+      <c r="C37" s="75" t="s">
         <v>19</v>
       </c>
-      <c r="D37" s="56"/>
-      <c r="E37" s="56"/>
-      <c r="F37" s="56"/>
-      <c r="G37" s="56"/>
-      <c r="H37" s="56"/>
-      <c r="I37" s="56"/>
-      <c r="J37" s="56"/>
-      <c r="K37" s="56"/>
-      <c r="L37" s="56"/>
-      <c r="M37" s="56"/>
-      <c r="N37" s="56"/>
-      <c r="O37" s="56"/>
+      <c r="D37" s="75"/>
+      <c r="E37" s="75"/>
+      <c r="F37" s="75"/>
+      <c r="G37" s="75"/>
+      <c r="H37" s="75"/>
+      <c r="I37" s="75"/>
+      <c r="J37" s="75"/>
+      <c r="K37" s="75"/>
+      <c r="L37" s="75"/>
+      <c r="M37" s="75"/>
+      <c r="N37" s="75"/>
+      <c r="O37" s="75"/>
     </row>
     <row r="38" spans="3:15" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="C38" s="56"/>
-      <c r="D38" s="56"/>
-      <c r="E38" s="56"/>
-      <c r="F38" s="56"/>
-      <c r="G38" s="56"/>
-      <c r="H38" s="56"/>
-      <c r="I38" s="56"/>
-      <c r="J38" s="56"/>
-      <c r="K38" s="56"/>
-      <c r="L38" s="56"/>
-      <c r="M38" s="56"/>
-      <c r="N38" s="56"/>
-      <c r="O38" s="56"/>
+      <c r="C38" s="75"/>
+      <c r="D38" s="75"/>
+      <c r="E38" s="75"/>
+      <c r="F38" s="75"/>
+      <c r="G38" s="75"/>
+      <c r="H38" s="75"/>
+      <c r="I38" s="75"/>
+      <c r="J38" s="75"/>
+      <c r="K38" s="75"/>
+      <c r="L38" s="75"/>
+      <c r="M38" s="75"/>
+      <c r="N38" s="75"/>
+      <c r="O38" s="75"/>
     </row>
     <row r="39" spans="3:15" customFormat="1" x14ac:dyDescent="0.3">
       <c r="G39" s="1"/>
@@ -2368,92 +2368,92 @@
       <c r="O41" s="20"/>
     </row>
     <row r="42" spans="3:15" customFormat="1" ht="23.4" x14ac:dyDescent="0.45">
-      <c r="C42" s="71" t="s">
+      <c r="C42" s="76" t="s">
         <v>20</v>
       </c>
-      <c r="D42" s="72"/>
-      <c r="E42" s="72"/>
-      <c r="F42" s="72"/>
-      <c r="G42" s="72"/>
-      <c r="H42" s="72"/>
-      <c r="I42" s="72"/>
-      <c r="J42" s="72"/>
-      <c r="K42" s="72"/>
-      <c r="L42" s="72"/>
-      <c r="M42" s="72"/>
-      <c r="N42" s="72"/>
-      <c r="O42" s="73"/>
+      <c r="D42" s="77"/>
+      <c r="E42" s="77"/>
+      <c r="F42" s="77"/>
+      <c r="G42" s="77"/>
+      <c r="H42" s="77"/>
+      <c r="I42" s="77"/>
+      <c r="J42" s="77"/>
+      <c r="K42" s="77"/>
+      <c r="L42" s="77"/>
+      <c r="M42" s="77"/>
+      <c r="N42" s="77"/>
+      <c r="O42" s="78"/>
     </row>
     <row r="43" spans="3:15" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="C43" s="61" t="s">
+      <c r="C43" s="68" t="s">
         <v>4</v>
       </c>
-      <c r="D43" s="62"/>
-      <c r="E43" s="74"/>
-      <c r="F43" s="74"/>
-      <c r="G43" s="74"/>
-      <c r="H43" s="74"/>
-      <c r="I43" s="74"/>
-      <c r="J43" s="74"/>
-      <c r="K43" s="74"/>
-      <c r="L43" s="74"/>
-      <c r="M43" s="74"/>
-      <c r="N43" s="74"/>
-      <c r="O43" s="74"/>
+      <c r="D43" s="69"/>
+      <c r="E43" s="66"/>
+      <c r="F43" s="66"/>
+      <c r="G43" s="66"/>
+      <c r="H43" s="66"/>
+      <c r="I43" s="66"/>
+      <c r="J43" s="66"/>
+      <c r="K43" s="66"/>
+      <c r="L43" s="66"/>
+      <c r="M43" s="66"/>
+      <c r="N43" s="66"/>
+      <c r="O43" s="66"/>
     </row>
     <row r="44" spans="3:15" x14ac:dyDescent="0.3">
-      <c r="C44" s="61" t="s">
+      <c r="C44" s="68" t="s">
         <v>21</v>
       </c>
-      <c r="D44" s="62"/>
-      <c r="E44" s="63"/>
-      <c r="F44" s="63"/>
-      <c r="G44" s="63"/>
+      <c r="D44" s="69"/>
+      <c r="E44" s="70"/>
+      <c r="F44" s="70"/>
+      <c r="G44" s="70"/>
       <c r="O44" s="21"/>
     </row>
     <row r="45" spans="3:15" x14ac:dyDescent="0.3">
-      <c r="C45" s="61" t="s">
+      <c r="C45" s="68" t="s">
         <v>22</v>
       </c>
-      <c r="D45" s="62"/>
-      <c r="E45" s="63"/>
-      <c r="F45" s="63"/>
-      <c r="G45" s="63"/>
+      <c r="D45" s="69"/>
+      <c r="E45" s="70"/>
+      <c r="F45" s="70"/>
+      <c r="G45" s="70"/>
       <c r="O45" s="21"/>
     </row>
     <row r="46" spans="3:15" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="C46" s="61" t="s">
+      <c r="C46" s="68" t="s">
         <v>23</v>
       </c>
-      <c r="D46" s="62"/>
-      <c r="E46" s="64"/>
-      <c r="F46" s="64"/>
-      <c r="G46" s="64"/>
-      <c r="H46" s="64"/>
-      <c r="I46" s="64"/>
-      <c r="J46" s="64"/>
-      <c r="K46" s="64"/>
-      <c r="L46" s="64"/>
-      <c r="M46" s="64"/>
-      <c r="N46" s="64"/>
-      <c r="O46" s="64"/>
+      <c r="D46" s="69"/>
+      <c r="E46" s="60"/>
+      <c r="F46" s="60"/>
+      <c r="G46" s="60"/>
+      <c r="H46" s="60"/>
+      <c r="I46" s="60"/>
+      <c r="J46" s="60"/>
+      <c r="K46" s="60"/>
+      <c r="L46" s="60"/>
+      <c r="M46" s="60"/>
+      <c r="N46" s="60"/>
+      <c r="O46" s="60"/>
     </row>
     <row r="47" spans="3:15" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="C47" s="61" t="s">
+      <c r="C47" s="68" t="s">
         <v>24</v>
       </c>
-      <c r="D47" s="62"/>
-      <c r="E47" s="64"/>
-      <c r="F47" s="64"/>
-      <c r="G47" s="64"/>
-      <c r="H47" s="64"/>
-      <c r="I47" s="64"/>
-      <c r="J47" s="64"/>
-      <c r="K47" s="64"/>
-      <c r="L47" s="64"/>
-      <c r="M47" s="64"/>
-      <c r="N47" s="64"/>
-      <c r="O47" s="64"/>
+      <c r="D47" s="69"/>
+      <c r="E47" s="60"/>
+      <c r="F47" s="60"/>
+      <c r="G47" s="60"/>
+      <c r="H47" s="60"/>
+      <c r="I47" s="60"/>
+      <c r="J47" s="60"/>
+      <c r="K47" s="60"/>
+      <c r="L47" s="60"/>
+      <c r="M47" s="60"/>
+      <c r="N47" s="60"/>
+      <c r="O47" s="60"/>
     </row>
     <row r="48" spans="3:15" x14ac:dyDescent="0.3">
       <c r="C48" s="22" t="s">
@@ -2621,12 +2621,12 @@
         <v>37</v>
       </c>
       <c r="D59"/>
-      <c r="E59" s="52"/>
-      <c r="F59" s="52"/>
-      <c r="G59" s="52"/>
-      <c r="H59" s="52"/>
-      <c r="I59" s="52"/>
-      <c r="J59" s="52"/>
+      <c r="E59" s="79"/>
+      <c r="F59" s="79"/>
+      <c r="G59" s="79"/>
+      <c r="H59" s="79"/>
+      <c r="I59" s="79"/>
+      <c r="J59" s="79"/>
       <c r="O59" s="21"/>
     </row>
     <row r="60" spans="3:18" x14ac:dyDescent="0.3">
@@ -2634,23 +2634,23 @@
         <v>38</v>
       </c>
       <c r="D60"/>
-      <c r="E60" s="52" t="s">
+      <c r="E60" s="79" t="s">
         <v>39</v>
       </c>
-      <c r="F60" s="52"/>
-      <c r="G60" s="52"/>
-      <c r="H60" s="52"/>
-      <c r="I60" s="52"/>
-      <c r="J60" s="52"/>
+      <c r="F60" s="79"/>
+      <c r="G60" s="79"/>
+      <c r="H60" s="79"/>
+      <c r="I60" s="79"/>
+      <c r="J60" s="79"/>
       <c r="O60" s="21"/>
     </row>
     <row r="61" spans="3:18" ht="35.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C61" s="53" t="s">
+      <c r="C61" s="80" t="s">
         <v>40</v>
       </c>
-      <c r="D61" s="54"/>
-      <c r="E61" s="52"/>
-      <c r="F61" s="52"/>
+      <c r="D61" s="81"/>
+      <c r="E61" s="79"/>
+      <c r="F61" s="79"/>
       <c r="O61" s="21"/>
       <c r="R61" s="4" t="s">
         <v>41</v>
@@ -2675,57 +2675,57 @@
       </c>
     </row>
     <row r="63" spans="3:18" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="C63" s="55" t="s">
+      <c r="C63" s="82" t="s">
         <v>42</v>
       </c>
-      <c r="D63" s="56"/>
-      <c r="E63" s="56"/>
-      <c r="F63" s="56"/>
-      <c r="G63" s="56"/>
-      <c r="H63" s="56"/>
-      <c r="I63" s="56"/>
-      <c r="J63" s="56"/>
-      <c r="K63" s="56"/>
-      <c r="L63" s="56"/>
-      <c r="M63" s="56"/>
-      <c r="N63" s="56"/>
-      <c r="O63" s="57"/>
+      <c r="D63" s="75"/>
+      <c r="E63" s="75"/>
+      <c r="F63" s="75"/>
+      <c r="G63" s="75"/>
+      <c r="H63" s="75"/>
+      <c r="I63" s="75"/>
+      <c r="J63" s="75"/>
+      <c r="K63" s="75"/>
+      <c r="L63" s="75"/>
+      <c r="M63" s="75"/>
+      <c r="N63" s="75"/>
+      <c r="O63" s="83"/>
       <c r="R63" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="64" spans="3:18" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="C64" s="55"/>
-      <c r="D64" s="56"/>
-      <c r="E64" s="56"/>
-      <c r="F64" s="56"/>
-      <c r="G64" s="56"/>
-      <c r="H64" s="56"/>
-      <c r="I64" s="56"/>
-      <c r="J64" s="56"/>
-      <c r="K64" s="56"/>
-      <c r="L64" s="56"/>
-      <c r="M64" s="56"/>
-      <c r="N64" s="56"/>
-      <c r="O64" s="57"/>
+      <c r="C64" s="82"/>
+      <c r="D64" s="75"/>
+      <c r="E64" s="75"/>
+      <c r="F64" s="75"/>
+      <c r="G64" s="75"/>
+      <c r="H64" s="75"/>
+      <c r="I64" s="75"/>
+      <c r="J64" s="75"/>
+      <c r="K64" s="75"/>
+      <c r="L64" s="75"/>
+      <c r="M64" s="75"/>
+      <c r="N64" s="75"/>
+      <c r="O64" s="83"/>
       <c r="R64" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="65" spans="3:18" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="C65" s="58"/>
-      <c r="D65" s="59"/>
-      <c r="E65" s="59"/>
-      <c r="F65" s="59"/>
-      <c r="G65" s="59"/>
-      <c r="H65" s="59"/>
-      <c r="I65" s="59"/>
-      <c r="J65" s="59"/>
-      <c r="K65" s="59"/>
-      <c r="L65" s="59"/>
-      <c r="M65" s="59"/>
-      <c r="N65" s="59"/>
-      <c r="O65" s="60"/>
+      <c r="C65" s="84"/>
+      <c r="D65" s="85"/>
+      <c r="E65" s="85"/>
+      <c r="F65" s="85"/>
+      <c r="G65" s="85"/>
+      <c r="H65" s="85"/>
+      <c r="I65" s="85"/>
+      <c r="J65" s="85"/>
+      <c r="K65" s="85"/>
+      <c r="L65" s="85"/>
+      <c r="M65" s="85"/>
+      <c r="N65" s="85"/>
+      <c r="O65" s="86"/>
       <c r="R65" t="s">
         <v>45</v>
       </c>
@@ -2756,21 +2756,17 @@
     </row>
   </sheetData>
   <mergeCells count="40">
-    <mergeCell ref="C11:O11"/>
-    <mergeCell ref="C14:D14"/>
-    <mergeCell ref="E14:O14"/>
-    <mergeCell ref="C15:D15"/>
-    <mergeCell ref="E15:O15"/>
-    <mergeCell ref="C22:O23"/>
-    <mergeCell ref="C25:D25"/>
-    <mergeCell ref="C26:D26"/>
-    <mergeCell ref="C16:D16"/>
-    <mergeCell ref="E16:O16"/>
-    <mergeCell ref="C17:D17"/>
-    <mergeCell ref="E17:O17"/>
-    <mergeCell ref="C18:D19"/>
-    <mergeCell ref="E19:O19"/>
-    <mergeCell ref="E20:O20"/>
+    <mergeCell ref="E59:J59"/>
+    <mergeCell ref="E60:J60"/>
+    <mergeCell ref="C61:D61"/>
+    <mergeCell ref="E61:F61"/>
+    <mergeCell ref="C63:O65"/>
+    <mergeCell ref="C45:D45"/>
+    <mergeCell ref="E45:G45"/>
+    <mergeCell ref="C46:D46"/>
+    <mergeCell ref="E46:O46"/>
+    <mergeCell ref="C47:D47"/>
+    <mergeCell ref="E47:O47"/>
     <mergeCell ref="C44:D44"/>
     <mergeCell ref="E44:G44"/>
     <mergeCell ref="C27:D27"/>
@@ -2785,17 +2781,21 @@
     <mergeCell ref="C43:D43"/>
     <mergeCell ref="E43:O43"/>
     <mergeCell ref="C28:D28"/>
-    <mergeCell ref="C45:D45"/>
-    <mergeCell ref="E45:G45"/>
-    <mergeCell ref="C46:D46"/>
-    <mergeCell ref="E46:O46"/>
-    <mergeCell ref="C47:D47"/>
-    <mergeCell ref="E47:O47"/>
-    <mergeCell ref="E59:J59"/>
-    <mergeCell ref="E60:J60"/>
-    <mergeCell ref="C61:D61"/>
-    <mergeCell ref="E61:F61"/>
-    <mergeCell ref="C63:O65"/>
+    <mergeCell ref="C22:O23"/>
+    <mergeCell ref="C25:D25"/>
+    <mergeCell ref="C26:D26"/>
+    <mergeCell ref="C16:D16"/>
+    <mergeCell ref="E16:O16"/>
+    <mergeCell ref="C17:D17"/>
+    <mergeCell ref="E17:O17"/>
+    <mergeCell ref="C18:D19"/>
+    <mergeCell ref="E19:O19"/>
+    <mergeCell ref="E20:O20"/>
+    <mergeCell ref="C11:O11"/>
+    <mergeCell ref="C14:D14"/>
+    <mergeCell ref="E14:O14"/>
+    <mergeCell ref="C15:D15"/>
+    <mergeCell ref="E15:O15"/>
   </mergeCells>
   <dataValidations count="2">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E60:J60" xr:uid="{EED16A01-C090-44A9-A7D6-FC173323C962}">

</xml_diff>